<commit_message>
Add author byline and contact card; fix clipped hero descender
- Byline (James Pieter Djibu, BSc Economics, Nagoya University, Class of 2028) on the report
  front page, page footers and disclosures, the Excel cover, website hero, README and portfolio summary
- Website: Contact section with email, LinkedIn and copy-to-clipboard email; Contact nav link
- Website: text-reveal mask no longer clips descenders (the p in Corporation)
- src/author.py holds author details for the report and model
</commit_message>
<xml_diff>
--- a/model/Makita_6586_model.xlsx
+++ b/model/Makita_6586_model.xlsx
@@ -33,9 +33,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="604" uniqueCount="434">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="605" uniqueCount="435">
   <si>
     <t xml:space="preserve">Makita Corporation (6586 JP): initiation model</t>
+  </si>
+  <si>
+    <t xml:space="preserve">By James Pieter Djibu, BSc Economics, Nagoya University, Class of 2028 (jamespieter16@gmail.com)</t>
   </si>
   <si>
     <t xml:space="preserve">Student research project, not investment advice. IFRS, JPY m, FY ends 31 March.</t>
@@ -1385,17 +1388,17 @@
       <charset val="1"/>
     </font>
     <font>
-      <i val="true"/>
+      <b val="true"/>
       <sz val="9"/>
-      <color rgb="FF5C5C5C"/>
+      <color theme="1"/>
       <name val="Arial"/>
       <family val="2"/>
       <charset val="1"/>
     </font>
     <font>
-      <b val="true"/>
+      <i val="true"/>
       <sz val="9"/>
-      <color theme="1"/>
+      <color rgb="FF5C5C5C"/>
       <name val="Arial"/>
       <family val="2"/>
       <charset val="1"/>
@@ -1565,7 +1568,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1593,7 +1596,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="166" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1605,7 +1608,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="167" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1613,7 +1616,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="168" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1621,7 +1624,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="169" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="169" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1637,7 +1640,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="170" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="170" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1661,7 +1664,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="166" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1685,7 +1688,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="170" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="170" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1945,7 +1948,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="B2:C21"/>
+  <dimension ref="B2:C22"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="4.71"/>
@@ -1964,119 +1967,124 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B5" s="3" t="s">
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B4" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="C5" s="4" t="str">
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B6" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C6" s="4" t="str">
         <f aca="false">Assumptions!E4</f>
         <v>Base</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B6" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="C6" s="4" t="str">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B7" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C7" s="4" t="str">
         <f aca="false">DCF!$D$62</f>
         <v>HOLD</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B7" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="C7" s="5" t="n">
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B8" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C8" s="5" t="n">
         <f aca="false">DCF!$D$58</f>
         <v>5850</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B8" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="C8" s="6" t="n">
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B9" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C9" s="6" t="n">
         <f aca="false">Assumptions!$D$85</f>
         <v>5253</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B9" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="C9" s="7" t="n">
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B10" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C10" s="7" t="n">
         <f aca="false">DCF!$D$60</f>
         <v>0.113649343232439</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B10" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="C10" s="6" t="n">
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B11" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C11" s="6" t="n">
         <f aca="false">DCF!$D$41</f>
         <v>5487.79158757565</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B11" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="C11" s="6" t="n">
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B12" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C12" s="6" t="n">
         <f aca="false">DCF!$D$50</f>
         <v>5561.06710554546</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B12" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="C12" s="7" t="n">
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B13" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C13" s="7" t="n">
         <f aca="false">Assumptions!$D$101</f>
         <v>0.0883738674377037</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B13" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="C13" s="7" t="n">
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B14" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C14" s="7" t="n">
         <f aca="false">Assumptions!$D$96</f>
         <v>0.089380336044146</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B14" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="C14" s="4" t="str">
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B15" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C15" s="4" t="str">
         <f aca="false">Checks!$C$25</f>
         <v>ALL CHECKS PASS</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B17" s="2" t="s">
-        <v>12</v>
-      </c>
-    </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B18" s="2" t="s">
+      <c r="B18" s="3" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B19" s="2" t="s">
+      <c r="B19" s="3" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B20" s="2" t="s">
+      <c r="B20" s="3" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B21" s="2" t="s">
+      <c r="B21" s="3" t="s">
         <v>16</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B22" s="3" t="s">
+        <v>17</v>
       </c>
     </row>
   </sheetData>
@@ -2105,32 +2113,32 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
-        <v>392</v>
+      <c r="A2" s="3" t="s">
+        <v>393</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="9" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="B4" s="9"/>
       <c r="C4" s="9" t="s">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>395</v>
+        <v>396</v>
       </c>
       <c r="E4" s="9" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="13" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="C5" s="6" t="n">
         <f aca="false">MIN(Sensitivity!$D$7:$F$9)</f>
@@ -2140,13 +2148,13 @@
         <f aca="false">MAX(Sensitivity!$D$7:$F$9)</f>
         <v>5930.17986608343</v>
       </c>
-      <c r="E5" s="2" t="s">
-        <v>398</v>
+      <c r="E5" s="3" t="s">
+        <v>399</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="13" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="C6" s="6" t="n">
         <f aca="false">MIN(Sensitivity!$D$15:$F$17)</f>
@@ -2156,13 +2164,13 @@
         <f aca="false">MAX(Sensitivity!$D$15:$F$17)</f>
         <v>6069.05001089495</v>
       </c>
-      <c r="E6" s="2" t="s">
-        <v>400</v>
+      <c r="E6" s="3" t="s">
+        <v>401</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="13" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="C7" s="6" t="n">
         <f aca="false">Comps!$D$35</f>
@@ -2172,13 +2180,13 @@
         <f aca="false">Comps!$D$37</f>
         <v>8975.49876670716</v>
       </c>
-      <c r="E7" s="2" t="s">
-        <v>402</v>
+      <c r="E7" s="3" t="s">
+        <v>403</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="13" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="C8" s="6" t="n">
         <f aca="false">Comps!$D$36</f>
@@ -2188,13 +2196,13 @@
         <f aca="false">Comps!$D$38</f>
         <v>9176.48744354829</v>
       </c>
-      <c r="E8" s="2" t="s">
-        <v>402</v>
+      <c r="E8" s="3" t="s">
+        <v>403</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="13" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="C9" s="6" t="n">
         <f aca="false">Comps!$D$39</f>
@@ -2204,13 +2212,13 @@
         <f aca="false">Comps!$D$40</f>
         <v>6931.8996974237</v>
       </c>
-      <c r="E9" s="2" t="s">
-        <v>405</v>
+      <c r="E9" s="3" t="s">
+        <v>406</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="13" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="C10" s="25" t="n">
         <v>4203</v>
@@ -2218,13 +2226,13 @@
       <c r="D10" s="25" t="n">
         <v>6106</v>
       </c>
-      <c r="E10" s="2" t="s">
-        <v>407</v>
+      <c r="E10" s="3" t="s">
+        <v>408</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="3" t="s">
-        <v>320</v>
+      <c r="A12" s="2" t="s">
+        <v>321</v>
       </c>
       <c r="C12" s="6" t="n">
         <f aca="false">Assumptions!$D$85</f>
@@ -2232,8 +2240,8 @@
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="3" t="s">
-        <v>408</v>
+      <c r="A13" s="2" t="s">
+        <v>409</v>
       </c>
       <c r="C13" s="5" t="n">
         <f aca="false">DCF!$D$58</f>
@@ -2266,56 +2274,56 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
-        <v>409</v>
+      <c r="A2" s="3" t="s">
+        <v>410</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="9" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="B4" s="9"/>
       <c r="C4" s="10" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D4" s="10" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="E4" s="10" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="F4" s="10" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="G4" s="10" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="H4" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="I4" s="10" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="J4" s="10" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="K4" s="10" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="L4" s="10" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="M4" s="9" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="13" t="s">
-        <v>411</v>
+        <v>412</v>
       </c>
       <c r="C5" s="36" t="b">
         <f aca="false">ABS(BS!C36)&lt;=2</f>
@@ -2357,13 +2365,13 @@
         <f aca="false">ABS(BS!L36-BS!G36)&lt;0.5</f>
         <v>1</v>
       </c>
-      <c r="M5" s="2" t="s">
-        <v>412</v>
+      <c r="M5" s="3" t="s">
+        <v>413</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="13" t="s">
-        <v>413</v>
+        <v>414</v>
       </c>
       <c r="C6" s="36" t="b">
         <f aca="false">ABS(CF!C35-BS!C7)&lt;=2</f>
@@ -2408,7 +2416,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="13" t="s">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="H7" s="36" t="b">
         <f aca="false">ABS(CF!H34-BS!G7)&lt;0.5</f>
@@ -2433,7 +2441,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="13" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="C8" s="36" t="b">
         <f aca="false">ABS(Drivers!C31-IS!C5)&lt;=2</f>
@@ -2475,13 +2483,13 @@
         <f aca="false">ABS(Drivers!L31-IS!L5)&lt;0.5</f>
         <v>1</v>
       </c>
-      <c r="M8" s="2" t="s">
-        <v>416</v>
+      <c r="M8" s="3" t="s">
+        <v>417</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="13" t="s">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="C9" s="36" t="b">
         <f aca="false">ABS(IS!C18-CF!C7)&lt;=2</f>
@@ -2526,7 +2534,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="13" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="H10" s="36" t="b">
         <f aca="false">ABS(BS!H29-BS!G29-IS!H20-CF!H24)&lt;0.5</f>
@@ -2551,7 +2559,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="13" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="H11" s="36" t="b">
         <f aca="false">ABS(DCF!H7-IS!H11)&lt;0.5</f>
@@ -2576,7 +2584,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="13" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="H12" s="36" t="b">
         <f aca="false">ABS(DCF!H11-CF!H19)&lt;0.5</f>
@@ -2601,7 +2609,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="13" t="s">
-        <v>421</v>
+        <v>422</v>
       </c>
       <c r="H13" s="36" t="b">
         <f aca="false">ABS(DCF!H12-(CF!H11+CF!H12+CF!H13+CF!H14))&lt;0.5</f>
@@ -2626,7 +2634,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="13" t="s">
-        <v>422</v>
+        <v>423</v>
       </c>
       <c r="H14" s="36" t="b">
         <f aca="false">ABS(-DCF!H8/DCF!H7-Assumptions!$G$70)&lt;0.0001</f>
@@ -2651,7 +2659,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="13" t="s">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="H15" s="36" t="b">
         <f aca="false">ABS(CF!H26+CF!H9)&lt;0.5</f>
@@ -2676,7 +2684,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="13" t="s">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="C16" s="36" t="b">
         <f aca="false">ABS(Assumptions!$D$100+Assumptions!$D$99-1)&lt;0.000001</f>
@@ -2685,7 +2693,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="13" t="s">
-        <v>425</v>
+        <v>426</v>
       </c>
       <c r="C17" s="36" t="b">
         <f aca="false">DCF!$D$28&lt;DCF!$D$27</f>
@@ -2694,7 +2702,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="13" t="s">
-        <v>426</v>
+        <v>427</v>
       </c>
       <c r="C18" s="36" t="b">
         <f aca="false">DCF!$D$28&lt;=Assumptions!$D$87</f>
@@ -2703,7 +2711,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="13" t="s">
-        <v>427</v>
+        <v>428</v>
       </c>
       <c r="C19" s="36" t="b">
         <f aca="false">DCF!$D$51&lt;=Assumptions!$D$87</f>
@@ -2712,7 +2720,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="13" t="s">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="C20" s="36" t="b">
         <f aca="false">ABS(Sensitivity!E8-DCF!$D$41)&lt;0.01</f>
@@ -2721,7 +2729,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="13" t="s">
-        <v>429</v>
+        <v>430</v>
       </c>
       <c r="C21" s="36" t="b">
         <f aca="false">ABS(Sensitivity!E16-DCF!$D$50)&lt;0.01</f>
@@ -2730,7 +2738,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="13" t="s">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="C22" s="36" t="b">
         <f aca="false">OR(Scenario=1,Scenario=2,Scenario=3)</f>
@@ -2739,7 +2747,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="13" t="s">
-        <v>431</v>
+        <v>432</v>
       </c>
       <c r="C23" s="36" t="b">
         <f aca="false">AND(DCF!H19&gt;0,DCF!H19&lt;=1)</f>
@@ -2747,15 +2755,15 @@
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="3" t="s">
-        <v>432</v>
+      <c r="A25" s="2" t="s">
+        <v>433</v>
       </c>
       <c r="C25" s="8" t="str">
         <f aca="false">IF(AND(C5,D5,E5,F5,G5,H5,I5,J5,K5,L5,C6,D6,E6,F6,G6,H6,I6,J6,K6,L6,H7,I7,J7,K7,L7,C8,D8,E8,F8,G8,H8,I8,J8,K8,L8,C9,D9,E9,F9,G9,H9,I9,J9,K9,L9,H10,I10,J10,K10,L10,H11,I11,J11,K11,L11,H12,I12,J12,K12,L12,H13,I13,J13,K13,L13,H14,I14,J14,K14,L14,H15,I15,J15,K15,L15,C16,C17,C18,C19,C20,C21,C22,C23),"ALL CHECKS PASS","CHECK FAILURES")</f>
         <v>ALL CHECKS PASS</v>
       </c>
-      <c r="E25" s="2" t="s">
-        <v>433</v>
+      <c r="E25" s="3" t="s">
+        <v>434</v>
       </c>
     </row>
   </sheetData>
@@ -2784,17 +2792,17 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
-        <v>18</v>
+      <c r="A2" s="3" t="s">
+        <v>19</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="3" t="s">
-        <v>19</v>
+      <c r="A4" s="2" t="s">
+        <v>20</v>
       </c>
       <c r="D4" s="8" t="n">
         <v>1</v>
@@ -2806,49 +2814,49 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="9" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B6" s="9"/>
       <c r="C6" s="10" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D6" s="10" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="E6" s="10" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="F6" s="10" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="G6" s="10" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="H6" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="I6" s="10" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="J6" s="10" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="K6" s="10" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="L6" s="10" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="M6" s="9" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="3" t="s">
-        <v>32</v>
+      <c r="A7" s="2" t="s">
+        <v>33</v>
       </c>
       <c r="B7" s="11" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="H7" s="12" t="n">
         <f aca="false">CHOOSE(Scenario,H8,H9,H10)</f>
@@ -2870,13 +2878,13 @@
         <f aca="false">CHOOSE(Scenario,L8,L9,L10)</f>
         <v>0.03</v>
       </c>
-      <c r="M7" s="2" t="s">
-        <v>34</v>
+      <c r="M7" s="3" t="s">
+        <v>35</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="13" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="H8" s="14" t="n">
         <v>0</v>
@@ -2896,7 +2904,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="13" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="H9" s="14" t="n">
         <v>0.02</v>
@@ -2916,7 +2924,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="13" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="H10" s="14" t="n">
         <v>-0.03</v>
@@ -2935,11 +2943,11 @@
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="3" t="s">
-        <v>38</v>
+      <c r="A11" s="2" t="s">
+        <v>39</v>
       </c>
       <c r="B11" s="11" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="H11" s="12" t="n">
         <f aca="false">CHOOSE(Scenario,H12,H13,H14)</f>
@@ -2961,13 +2969,13 @@
         <f aca="false">CHOOSE(Scenario,L12,L13,L14)</f>
         <v>0.015</v>
       </c>
-      <c r="M11" s="2" t="s">
-        <v>39</v>
+      <c r="M11" s="3" t="s">
+        <v>40</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="13" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="H12" s="14" t="n">
         <v>0.025</v>
@@ -2987,7 +2995,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="13" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="H13" s="14" t="n">
         <v>0.04</v>
@@ -3007,7 +3015,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="13" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="H14" s="14" t="n">
         <v>0</v>
@@ -3026,11 +3034,11 @@
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="3" t="s">
-        <v>40</v>
+      <c r="A15" s="2" t="s">
+        <v>41</v>
       </c>
       <c r="B15" s="11" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="H15" s="12" t="n">
         <f aca="false">CHOOSE(Scenario,H16,H17,H18)</f>
@@ -3052,13 +3060,13 @@
         <f aca="false">CHOOSE(Scenario,L16,L17,L18)</f>
         <v>0.03</v>
       </c>
-      <c r="M15" s="2" t="s">
-        <v>41</v>
+      <c r="M15" s="3" t="s">
+        <v>42</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="13" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="H16" s="14" t="n">
         <v>0.03</v>
@@ -3078,7 +3086,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="13" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="H17" s="14" t="n">
         <v>0.06</v>
@@ -3098,7 +3106,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="13" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="H18" s="14" t="n">
         <v>-0.03</v>
@@ -3117,11 +3125,11 @@
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="3" t="s">
-        <v>42</v>
+      <c r="A19" s="2" t="s">
+        <v>43</v>
       </c>
       <c r="B19" s="11" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="H19" s="12" t="n">
         <f aca="false">CHOOSE(Scenario,H20,H21,H22)</f>
@@ -3143,13 +3151,13 @@
         <f aca="false">CHOOSE(Scenario,L20,L21,L22)</f>
         <v>0.035</v>
       </c>
-      <c r="M19" s="2" t="s">
-        <v>43</v>
+      <c r="M19" s="3" t="s">
+        <v>44</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="13" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="H20" s="14" t="n">
         <v>0.02</v>
@@ -3169,7 +3177,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="13" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="H21" s="14" t="n">
         <v>0.04</v>
@@ -3189,7 +3197,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="13" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="H22" s="14" t="n">
         <v>-0.02</v>
@@ -3208,11 +3216,11 @@
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="3" t="s">
-        <v>44</v>
+      <c r="A23" s="2" t="s">
+        <v>45</v>
       </c>
       <c r="B23" s="11" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="H23" s="15" t="n">
         <f aca="false">CHOOSE(Scenario,H24,H25,H26)</f>
@@ -3234,13 +3242,13 @@
         <f aca="false">CHOOSE(Scenario,L24,L25,L26)</f>
         <v>157.82</v>
       </c>
-      <c r="M23" s="2" t="s">
-        <v>46</v>
+      <c r="M23" s="3" t="s">
+        <v>47</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="13" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="H24" s="16" t="n">
         <v>158.26</v>
@@ -3260,7 +3268,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="13" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="H25" s="16" t="n">
         <v>158.26</v>
@@ -3280,7 +3288,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="13" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="H26" s="16" t="n">
         <v>154.31</v>
@@ -3299,11 +3307,11 @@
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="3" t="s">
-        <v>47</v>
+      <c r="A27" s="2" t="s">
+        <v>48</v>
       </c>
       <c r="B27" s="11" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="H27" s="15" t="n">
         <f aca="false">CHOOSE(Scenario,H28,H29,H30)</f>
@@ -3325,13 +3333,13 @@
         <f aca="false">CHOOSE(Scenario,L28,L29,L30)</f>
         <v>176.03</v>
       </c>
-      <c r="M27" s="2" t="s">
-        <v>48</v>
+      <c r="M27" s="3" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="13" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="H28" s="16" t="n">
         <v>178.38</v>
@@ -3351,7 +3359,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="13" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="H29" s="16" t="n">
         <v>178.38</v>
@@ -3371,7 +3379,7 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="13" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="H30" s="16" t="n">
         <v>174.08</v>
@@ -3390,11 +3398,11 @@
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="3" t="s">
-        <v>49</v>
+      <c r="A31" s="2" t="s">
+        <v>50</v>
       </c>
       <c r="B31" s="11" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="H31" s="12" t="n">
         <f aca="false">CHOOSE(Scenario,H32,H33,H34)</f>
@@ -3416,13 +3424,13 @@
         <f aca="false">CHOOSE(Scenario,L32,L33,L34)</f>
         <v>0.365</v>
       </c>
-      <c r="M31" s="2" t="s">
-        <v>50</v>
+      <c r="M31" s="3" t="s">
+        <v>51</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="13" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="H32" s="14" t="n">
         <v>0.37</v>
@@ -3442,7 +3450,7 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="13" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="H33" s="14" t="n">
         <v>0.375</v>
@@ -3462,7 +3470,7 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="13" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="H34" s="14" t="n">
         <v>0.355</v>
@@ -3481,11 +3489,11 @@
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="3" t="s">
-        <v>51</v>
+      <c r="A35" s="2" t="s">
+        <v>52</v>
       </c>
       <c r="B35" s="11" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="H35" s="12" t="n">
         <f aca="false">CHOOSE(Scenario,H36,H37,H38)</f>
@@ -3507,13 +3515,13 @@
         <f aca="false">CHOOSE(Scenario,L36,L37,L38)</f>
         <v>0.225</v>
       </c>
-      <c r="M35" s="2" t="s">
-        <v>52</v>
+      <c r="M35" s="3" t="s">
+        <v>53</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="13" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="H36" s="14" t="n">
         <v>0.233</v>
@@ -3533,7 +3541,7 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="13" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="H37" s="14" t="n">
         <v>0.23</v>
@@ -3553,7 +3561,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="13" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="H38" s="14" t="n">
         <v>0.238</v>
@@ -3572,11 +3580,11 @@
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="3" t="s">
-        <v>53</v>
+      <c r="A39" s="2" t="s">
+        <v>54</v>
       </c>
       <c r="B39" s="11" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="H39" s="17" t="n">
         <f aca="false">CHOOSE(Scenario,H40,H41,H42)</f>
@@ -3598,13 +3606,13 @@
         <f aca="false">CHOOSE(Scenario,L40,L41,L42)</f>
         <v>57</v>
       </c>
-      <c r="M39" s="2" t="s">
-        <v>55</v>
+      <c r="M39" s="3" t="s">
+        <v>56</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="13" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="H40" s="18" t="n">
         <v>57</v>
@@ -3624,7 +3632,7 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="13" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="H41" s="18" t="n">
         <v>55</v>
@@ -3644,7 +3652,7 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="13" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="H42" s="18" t="n">
         <v>60</v>
@@ -3663,11 +3671,11 @@
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="3" t="s">
-        <v>56</v>
+      <c r="A43" s="2" t="s">
+        <v>57</v>
       </c>
       <c r="B43" s="11" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="H43" s="17" t="n">
         <f aca="false">CHOOSE(Scenario,H44,H45,H46)</f>
@@ -3689,13 +3697,13 @@
         <f aca="false">CHOOSE(Scenario,L44,L45,L46)</f>
         <v>255</v>
       </c>
-      <c r="M43" s="2" t="s">
-        <v>57</v>
+      <c r="M43" s="3" t="s">
+        <v>58</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="13" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="H44" s="18" t="n">
         <v>275</v>
@@ -3715,7 +3723,7 @@
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="13" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="H45" s="18" t="n">
         <v>270</v>
@@ -3735,7 +3743,7 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="13" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="H46" s="18" t="n">
         <v>290</v>
@@ -3754,11 +3762,11 @@
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A47" s="3" t="s">
-        <v>58</v>
+      <c r="A47" s="2" t="s">
+        <v>59</v>
       </c>
       <c r="B47" s="11" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="H47" s="17" t="n">
         <f aca="false">CHOOSE(Scenario,H48,H49,H50)</f>
@@ -3780,13 +3788,13 @@
         <f aca="false">CHOOSE(Scenario,L48,L49,L50)</f>
         <v>41</v>
       </c>
-      <c r="M47" s="2" t="s">
-        <v>59</v>
+      <c r="M47" s="3" t="s">
+        <v>60</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="13" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="H48" s="18" t="n">
         <v>41</v>
@@ -3806,7 +3814,7 @@
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="13" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="H49" s="18" t="n">
         <v>42</v>
@@ -3826,7 +3834,7 @@
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="13" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="H50" s="18" t="n">
         <v>39</v>
@@ -3845,11 +3853,11 @@
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A51" s="3" t="s">
-        <v>60</v>
+      <c r="A51" s="2" t="s">
+        <v>61</v>
       </c>
       <c r="B51" s="11" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="H51" s="12" t="n">
         <f aca="false">CHOOSE(Scenario,H52,H53,H54)</f>
@@ -3871,13 +3879,13 @@
         <f aca="false">CHOOSE(Scenario,L52,L53,L54)</f>
         <v>0.025</v>
       </c>
-      <c r="M51" s="2" t="s">
-        <v>61</v>
+      <c r="M51" s="3" t="s">
+        <v>62</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="13" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="H52" s="14" t="n">
         <v>0.025</v>
@@ -3897,7 +3905,7 @@
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="13" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="H53" s="14" t="n">
         <v>0.025</v>
@@ -3917,7 +3925,7 @@
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="13" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="H54" s="14" t="n">
         <v>0.025</v>
@@ -3936,11 +3944,11 @@
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A55" s="3" t="s">
-        <v>62</v>
+      <c r="A55" s="2" t="s">
+        <v>63</v>
       </c>
       <c r="B55" s="11" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="H55" s="12" t="n">
         <f aca="false">CHOOSE(Scenario,H56,H57,H58)</f>
@@ -3962,13 +3970,13 @@
         <f aca="false">CHOOSE(Scenario,L56,L57,L58)</f>
         <v>0.098</v>
       </c>
-      <c r="M55" s="2" t="s">
-        <v>63</v>
+      <c r="M55" s="3" t="s">
+        <v>64</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="13" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="H56" s="14" t="n">
         <v>0.098</v>
@@ -3988,7 +3996,7 @@
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="13" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="H57" s="14" t="n">
         <v>0.098</v>
@@ -4008,7 +4016,7 @@
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="13" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="H58" s="14" t="n">
         <v>0.098</v>
@@ -4027,11 +4035,11 @@
       </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A59" s="3" t="s">
-        <v>64</v>
+      <c r="A59" s="2" t="s">
+        <v>65</v>
       </c>
       <c r="B59" s="11" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="H59" s="12" t="n">
         <f aca="false">CHOOSE(Scenario,H60,H61,H62)</f>
@@ -4053,13 +4061,13 @@
         <f aca="false">CHOOSE(Scenario,L60,L61,L62)</f>
         <v>0.032</v>
       </c>
-      <c r="M59" s="2" t="s">
-        <v>65</v>
+      <c r="M59" s="3" t="s">
+        <v>66</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="13" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="H60" s="14" t="n">
         <v>0.036</v>
@@ -4079,7 +4087,7 @@
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="13" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="H61" s="14" t="n">
         <v>0.036</v>
@@ -4099,7 +4107,7 @@
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="13" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="H62" s="14" t="n">
         <v>0.033</v>
@@ -4118,11 +4126,11 @@
       </c>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A63" s="3" t="s">
-        <v>66</v>
+      <c r="A63" s="2" t="s">
+        <v>67</v>
       </c>
       <c r="B63" s="11" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="H63" s="19" t="n">
         <f aca="false">CHOOSE(Scenario,H64,H65,H66)</f>
@@ -4144,13 +4152,13 @@
         <f aca="false">CHOOSE(Scenario,L64,L65,L66)</f>
         <v>0</v>
       </c>
-      <c r="M63" s="2" t="s">
-        <v>68</v>
+      <c r="M63" s="3" t="s">
+        <v>69</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="13" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="H64" s="20" t="n">
         <v>0</v>
@@ -4170,7 +4178,7 @@
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="13" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="H65" s="20" t="n">
         <v>20000</v>
@@ -4190,7 +4198,7 @@
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="13" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="H66" s="20" t="n">
         <v>0</v>
@@ -4210,26 +4218,26 @@
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="21" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D69" s="10" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E69" s="10" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="F69" s="10" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="G69" s="10" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A70" s="13" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="D70" s="14" t="n">
         <v>0.27</v>
@@ -4244,13 +4252,13 @@
         <f aca="false">CHOOSE(Scenario,D70,E70,F70)</f>
         <v>0.27</v>
       </c>
-      <c r="M70" s="2" t="s">
-        <v>75</v>
+      <c r="M70" s="3" t="s">
+        <v>76</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A71" s="13" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="D71" s="14" t="n">
         <v>0.093</v>
@@ -4265,13 +4273,13 @@
         <f aca="false">CHOOSE(Scenario,D71,E71,F71)</f>
         <v>0.093</v>
       </c>
-      <c r="M71" s="2" t="s">
-        <v>77</v>
+      <c r="M71" s="3" t="s">
+        <v>78</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A72" s="13" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="D72" s="14" t="n">
         <v>0.0068</v>
@@ -4286,13 +4294,13 @@
         <f aca="false">CHOOSE(Scenario,D72,E72,F72)</f>
         <v>0.0068</v>
       </c>
-      <c r="M72" s="2" t="s">
-        <v>79</v>
+      <c r="M72" s="3" t="s">
+        <v>80</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A73" s="13" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D73" s="14" t="n">
         <v>0.018</v>
@@ -4307,13 +4315,13 @@
         <f aca="false">CHOOSE(Scenario,D73,E73,F73)</f>
         <v>0.018</v>
       </c>
-      <c r="M73" s="2" t="s">
-        <v>81</v>
+      <c r="M73" s="3" t="s">
+        <v>82</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A74" s="13" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="D74" s="20" t="n">
         <v>-1200</v>
@@ -4328,13 +4336,13 @@
         <f aca="false">CHOOSE(Scenario,D74,E74,F74)</f>
         <v>-1200</v>
       </c>
-      <c r="M74" s="2" t="s">
-        <v>83</v>
+      <c r="M74" s="3" t="s">
+        <v>84</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A75" s="13" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="D75" s="14" t="n">
         <v>0.001</v>
@@ -4349,13 +4357,13 @@
         <f aca="false">CHOOSE(Scenario,D75,E75,F75)</f>
         <v>0.001</v>
       </c>
-      <c r="M75" s="2" t="s">
-        <v>85</v>
+      <c r="M75" s="3" t="s">
+        <v>86</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A76" s="13" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="D76" s="14" t="n">
         <v>0.5</v>
@@ -4370,13 +4378,13 @@
         <f aca="false">CHOOSE(Scenario,D76,E76,F76)</f>
         <v>0.5</v>
       </c>
-      <c r="M76" s="2" t="s">
-        <v>87</v>
+      <c r="M76" s="3" t="s">
+        <v>88</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A77" s="13" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D77" s="20" t="n">
         <v>100000</v>
@@ -4391,13 +4399,13 @@
         <f aca="false">CHOOSE(Scenario,D77,E77,F77)</f>
         <v>100000</v>
       </c>
-      <c r="M77" s="2" t="s">
-        <v>89</v>
+      <c r="M77" s="3" t="s">
+        <v>90</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A78" s="13" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="D78" s="14" t="n">
         <v>0.02</v>
@@ -4412,13 +4420,13 @@
         <f aca="false">CHOOSE(Scenario,D78,E78,F78)</f>
         <v>0.02</v>
       </c>
-      <c r="M78" s="2" t="s">
-        <v>91</v>
+      <c r="M78" s="3" t="s">
+        <v>92</v>
       </c>
     </row>
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A79" s="13" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="D79" s="14" t="n">
         <v>0.12</v>
@@ -4433,13 +4441,13 @@
         <f aca="false">CHOOSE(Scenario,D79,E79,F79)</f>
         <v>0.12</v>
       </c>
-      <c r="M79" s="2" t="s">
-        <v>93</v>
+      <c r="M79" s="3" t="s">
+        <v>94</v>
       </c>
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A80" s="13" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="D80" s="22" t="n">
         <v>7.5</v>
@@ -4454,299 +4462,299 @@
         <f aca="false">CHOOSE(Scenario,D80,E80,F80)</f>
         <v>7.5</v>
       </c>
-      <c r="M80" s="2" t="s">
-        <v>95</v>
+      <c r="M80" s="3" t="s">
+        <v>96</v>
       </c>
     </row>
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A82" s="21" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
     </row>
     <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A83" s="13" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="D83" s="24" t="n">
         <v>46324</v>
       </c>
-      <c r="M83" s="2" t="s">
-        <v>98</v>
+      <c r="M83" s="3" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A84" s="13" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="D84" s="24" t="n">
         <v>46203</v>
       </c>
-      <c r="M84" s="2" t="s">
-        <v>100</v>
+      <c r="M84" s="3" t="s">
+        <v>101</v>
       </c>
     </row>
     <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A85" s="13" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="D85" s="25" t="n">
         <v>5253</v>
       </c>
-      <c r="M85" s="2" t="s">
-        <v>102</v>
+      <c r="M85" s="3" t="s">
+        <v>103</v>
       </c>
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A86" s="13" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D86" s="16" t="n">
         <v>257.655511</v>
       </c>
-      <c r="M86" s="2" t="s">
-        <v>104</v>
+      <c r="M86" s="3" t="s">
+        <v>105</v>
       </c>
     </row>
     <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A87" s="13" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="D87" s="14" t="n">
         <v>0.02867</v>
       </c>
-      <c r="M87" s="2" t="s">
-        <v>106</v>
+      <c r="M87" s="3" t="s">
+        <v>107</v>
       </c>
     </row>
     <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A88" s="13" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="D88" s="14" t="n">
         <v>0.0423</v>
       </c>
-      <c r="M88" s="2" t="s">
-        <v>108</v>
+      <c r="M88" s="3" t="s">
+        <v>109</v>
       </c>
     </row>
     <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A89" s="13" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="D89" s="14" t="n">
         <v>0.0119823576533909</v>
       </c>
-      <c r="M89" s="2" t="s">
-        <v>110</v>
+      <c r="M89" s="3" t="s">
+        <v>111</v>
       </c>
     </row>
     <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A90" s="13" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="D90" s="26" t="n">
         <v>1.10531271085682</v>
       </c>
-      <c r="M90" s="2" t="s">
-        <v>112</v>
+      <c r="M90" s="3" t="s">
+        <v>113</v>
       </c>
     </row>
     <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A91" s="13" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="D91" s="20" t="n">
         <v>21982</v>
       </c>
-      <c r="M91" s="2" t="s">
-        <v>114</v>
+      <c r="M91" s="3" t="s">
+        <v>115</v>
       </c>
     </row>
     <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A92" s="13" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="D92" s="27" t="n">
         <f aca="false">Assumptions!$D$85*Assumptions!$D$86</f>
         <v>1353464.399283</v>
       </c>
-      <c r="M92" s="2" t="s">
-        <v>116</v>
+      <c r="M92" s="3" t="s">
+        <v>117</v>
       </c>
     </row>
     <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A93" s="13" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="D93" s="7" t="n">
         <f aca="false">Assumptions!$D$91/Assumptions!$D$92</f>
         <v>0.0162412842270879</v>
       </c>
-      <c r="M93" s="2"/>
+      <c r="M93" s="3"/>
     </row>
     <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A94" s="13" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="D94" s="28" t="n">
         <f aca="false">Assumptions!$D$90*(1+(1-Assumptions!$G$70)*Assumptions!$D$93)</f>
         <v>1.11841745032151</v>
       </c>
-      <c r="M94" s="2" t="s">
-        <v>119</v>
+      <c r="M94" s="3" t="s">
+        <v>120</v>
       </c>
     </row>
     <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A95" s="13" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="D95" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="M95" s="2" t="s">
-        <v>121</v>
+      <c r="M95" s="3" t="s">
+        <v>122</v>
       </c>
     </row>
     <row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A96" s="13" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D96" s="7" t="n">
         <f aca="false">Assumptions!$D$87+Assumptions!$D$94*(Assumptions!$D$88+Assumptions!$D$89)+Assumptions!$D$95</f>
         <v>0.089380336044146</v>
       </c>
-      <c r="M96" s="2" t="s">
-        <v>122</v>
+      <c r="M96" s="3" t="s">
+        <v>123</v>
       </c>
     </row>
     <row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A97" s="13" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="D97" s="14" t="n">
         <v>0.0075</v>
       </c>
-      <c r="M97" s="2" t="s">
-        <v>124</v>
+      <c r="M97" s="3" t="s">
+        <v>125</v>
       </c>
     </row>
     <row r="98" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A98" s="13" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="D98" s="7" t="n">
         <f aca="false">(Assumptions!$D$87+Assumptions!$D$97)*(1-Assumptions!$G$70)</f>
         <v>0.0264041</v>
       </c>
-      <c r="M98" s="2"/>
+      <c r="M98" s="3"/>
     </row>
     <row r="99" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A99" s="13" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="D99" s="7" t="n">
         <f aca="false">Assumptions!$D$91/(Assumptions!$D$91+Assumptions!$D$92)</f>
         <v>0.0159817205610185</v>
       </c>
-      <c r="M99" s="2" t="s">
-        <v>127</v>
+      <c r="M99" s="3" t="s">
+        <v>128</v>
       </c>
     </row>
     <row r="100" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A100" s="13" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="D100" s="7" t="n">
         <f aca="false">1-Assumptions!$D$99</f>
         <v>0.984018279438982</v>
       </c>
-      <c r="M100" s="2"/>
+      <c r="M100" s="3"/>
     </row>
     <row r="101" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A101" s="13" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D101" s="29" t="n">
         <f aca="false">Assumptions!$D$100*Assumptions!$D$96+Assumptions!$D$99*Assumptions!$D$98</f>
         <v>0.0883738674377037</v>
       </c>
-      <c r="M101" s="2"/>
+      <c r="M101" s="3"/>
     </row>
     <row r="102" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A102" s="13" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="D102" s="20" t="n">
         <v>256364</v>
       </c>
-      <c r="M102" s="2" t="s">
-        <v>130</v>
+      <c r="M102" s="3" t="s">
+        <v>131</v>
       </c>
     </row>
     <row r="103" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A103" s="13" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="D103" s="20" t="n">
         <v>27921</v>
       </c>
-      <c r="M103" s="2" t="s">
-        <v>130</v>
+      <c r="M103" s="3" t="s">
+        <v>131</v>
       </c>
     </row>
     <row r="104" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A104" s="13" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="D104" s="20" t="n">
         <v>55562</v>
       </c>
-      <c r="M104" s="2" t="s">
-        <v>133</v>
+      <c r="M104" s="3" t="s">
+        <v>134</v>
       </c>
     </row>
     <row r="105" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A105" s="13" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="D105" s="20" t="n">
         <v>1604</v>
       </c>
-      <c r="M105" s="2" t="s">
-        <v>130</v>
+      <c r="M105" s="3" t="s">
+        <v>131</v>
       </c>
     </row>
     <row r="106" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A106" s="13" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="D106" s="20" t="n">
         <v>7432</v>
       </c>
-      <c r="M106" s="2" t="s">
-        <v>130</v>
+      <c r="M106" s="3" t="s">
+        <v>131</v>
       </c>
     </row>
     <row r="107" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A107" s="13" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="D107" s="20" t="n">
         <v>19104</v>
       </c>
-      <c r="M107" s="2" t="s">
-        <v>137</v>
+      <c r="M107" s="3" t="s">
+        <v>138</v>
       </c>
     </row>
     <row r="108" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A108" s="13" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="D108" s="25" t="n">
         <v>79</v>
       </c>
-      <c r="M108" s="2" t="s">
-        <v>139</v>
+      <c r="M108" s="3" t="s">
+        <v>140</v>
       </c>
     </row>
   </sheetData>
@@ -4781,61 +4789,61 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
-        <v>141</v>
+      <c r="A2" s="3" t="s">
+        <v>142</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="9" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="B4" s="9"/>
       <c r="C4" s="10" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D4" s="10" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="E4" s="10" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="F4" s="10" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="G4" s="10" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="H4" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="I4" s="10" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="J4" s="10" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="K4" s="10" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="L4" s="10" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="M4" s="9" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="21" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="13" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="B7" s="11"/>
       <c r="C7" s="16" t="n">
@@ -4873,13 +4881,13 @@
         <f aca="false">Assumptions!L23</f>
         <v>157.82</v>
       </c>
-      <c r="M7" s="2" t="s">
-        <v>145</v>
+      <c r="M7" s="3" t="s">
+        <v>146</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="13" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="B8" s="11"/>
       <c r="C8" s="16" t="n">
@@ -4920,12 +4928,12 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="21" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="13" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="B11" s="11"/>
       <c r="C11" s="20" t="n">
@@ -4963,13 +4971,13 @@
         <f aca="false">K11*(1+Assumptions!L7)*(L8/K8)</f>
         <v>440418.535909783</v>
       </c>
-      <c r="M11" s="2" t="s">
-        <v>149</v>
+      <c r="M11" s="3" t="s">
+        <v>150</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="13" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="B12" s="11"/>
       <c r="C12" s="7" t="str">
@@ -5015,7 +5023,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="13" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="B13" s="11"/>
       <c r="C13" s="7" t="str">
@@ -5058,18 +5066,18 @@
         <f aca="false">Assumptions!L7</f>
         <v>0.03</v>
       </c>
-      <c r="M13" s="2" t="s">
-        <v>152</v>
+      <c r="M13" s="3" t="s">
+        <v>153</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="21" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="13" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="B16" s="11"/>
       <c r="C16" s="20" t="n">
@@ -5107,13 +5115,13 @@
         <f aca="false">K16*(1+Assumptions!L11)</f>
         <v>145885.315417128</v>
       </c>
-      <c r="M16" s="2" t="s">
-        <v>149</v>
+      <c r="M16" s="3" t="s">
+        <v>150</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="13" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="B17" s="11"/>
       <c r="C17" s="7" t="str">
@@ -5159,7 +5167,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="13" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="B18" s="11"/>
       <c r="C18" s="7" t="str">
@@ -5202,18 +5210,18 @@
         <f aca="false">Assumptions!L11</f>
         <v>0.015</v>
       </c>
-      <c r="M18" s="2" t="s">
-        <v>152</v>
+      <c r="M18" s="3" t="s">
+        <v>153</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="21" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="13" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="B21" s="11"/>
       <c r="C21" s="20" t="n">
@@ -5251,13 +5259,13 @@
         <f aca="false">K21*(1+Assumptions!L15)*(L7/K7)</f>
         <v>95518.2503195515</v>
       </c>
-      <c r="M21" s="2" t="s">
-        <v>149</v>
+      <c r="M21" s="3" t="s">
+        <v>150</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="13" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="B22" s="11"/>
       <c r="C22" s="7" t="str">
@@ -5303,7 +5311,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="13" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="B23" s="11"/>
       <c r="C23" s="7" t="str">
@@ -5346,18 +5354,18 @@
         <f aca="false">Assumptions!L15</f>
         <v>0.03</v>
       </c>
-      <c r="M23" s="2" t="s">
-        <v>152</v>
+      <c r="M23" s="3" t="s">
+        <v>153</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="21" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="13" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="B26" s="11"/>
       <c r="C26" s="20" t="n">
@@ -5395,13 +5403,13 @@
         <f aca="false">K26*(1+Assumptions!L19)*(L7/K7)</f>
         <v>218725.635648361</v>
       </c>
-      <c r="M26" s="2" t="s">
-        <v>149</v>
+      <c r="M26" s="3" t="s">
+        <v>150</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="13" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="B27" s="11"/>
       <c r="C27" s="7" t="str">
@@ -5447,7 +5455,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="13" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="B28" s="11"/>
       <c r="C28" s="7" t="str">
@@ -5490,18 +5498,18 @@
         <f aca="false">Assumptions!L19</f>
         <v>0.035</v>
       </c>
-      <c r="M28" s="2" t="s">
-        <v>152</v>
+      <c r="M28" s="3" t="s">
+        <v>153</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="21" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="3" t="s">
-        <v>160</v>
+      <c r="A31" s="2" t="s">
+        <v>161</v>
       </c>
       <c r="B31" s="11"/>
       <c r="C31" s="19" t="n">
@@ -5547,7 +5555,7 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="13" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="B32" s="11"/>
       <c r="C32" s="7" t="str">
@@ -5593,7 +5601,7 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="13" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="B33" s="11"/>
       <c r="H33" s="7" t="n">
@@ -5616,8 +5624,8 @@
         <f aca="false">(L31-SUMPRODUCT(K11*(1+Assumptions!L7)+K16*(1+Assumptions!L11)+K21*(1+Assumptions!L15)+K26*(1+Assumptions!L19)))/K31</f>
         <v>0</v>
       </c>
-      <c r="M33" s="2" t="s">
-        <v>163</v>
+      <c r="M33" s="3" t="s">
+        <v>164</v>
       </c>
     </row>
   </sheetData>
@@ -5646,56 +5654,56 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
-        <v>165</v>
+      <c r="A2" s="3" t="s">
+        <v>166</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="9" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="B4" s="9"/>
       <c r="C4" s="10" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D4" s="10" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="E4" s="10" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="F4" s="10" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="G4" s="10" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="H4" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="I4" s="10" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="J4" s="10" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="K4" s="10" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="L4" s="10" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="M4" s="9" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="3" t="s">
-        <v>166</v>
+      <c r="A5" s="2" t="s">
+        <v>167</v>
       </c>
       <c r="B5" s="11"/>
       <c r="C5" s="31" t="n">
@@ -5733,13 +5741,13 @@
         <f aca="false">Drivers!L31</f>
         <v>900547.737294824</v>
       </c>
-      <c r="M5" s="2" t="s">
-        <v>167</v>
+      <c r="M5" s="3" t="s">
+        <v>168</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="13" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="B6" s="11"/>
       <c r="C6" s="7" t="str">
@@ -5785,7 +5793,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="13" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="B7" s="11"/>
       <c r="C7" s="20" t="n">
@@ -5825,8 +5833,8 @@
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="3" t="s">
-        <v>169</v>
+      <c r="A8" s="2" t="s">
+        <v>170</v>
       </c>
       <c r="B8" s="11"/>
       <c r="C8" s="19" t="n">
@@ -5872,7 +5880,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="13" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="B9" s="11"/>
       <c r="C9" s="7" t="n">
@@ -5918,7 +5926,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="13" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="B10" s="11"/>
       <c r="C10" s="20" t="n">
@@ -5958,8 +5966,8 @@
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="3" t="s">
-        <v>172</v>
+      <c r="A11" s="2" t="s">
+        <v>173</v>
       </c>
       <c r="B11" s="11"/>
       <c r="C11" s="19" t="n">
@@ -6005,7 +6013,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="13" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="B12" s="11"/>
       <c r="C12" s="7" t="n">
@@ -6051,7 +6059,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="13" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="B13" s="11"/>
       <c r="C13" s="20" t="n">
@@ -6089,13 +6097,13 @@
         <f aca="false">Assumptions!$G$73*(BS!K7+BS!K8)</f>
         <v>7938.27020653075</v>
       </c>
-      <c r="M13" s="2" t="s">
-        <v>175</v>
+      <c r="M13" s="3" t="s">
+        <v>176</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="13" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="B14" s="11"/>
       <c r="C14" s="20" t="n">
@@ -6135,8 +6143,8 @@
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="3" t="s">
-        <v>177</v>
+      <c r="A15" s="2" t="s">
+        <v>178</v>
       </c>
       <c r="B15" s="11"/>
       <c r="C15" s="19" t="n">
@@ -6182,7 +6190,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="13" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="B16" s="11"/>
       <c r="C16" s="20" t="n">
@@ -6223,7 +6231,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="13" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="B17" s="11"/>
       <c r="C17" s="7" t="n">
@@ -6268,8 +6276,8 @@
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="3" t="s">
-        <v>180</v>
+      <c r="A18" s="2" t="s">
+        <v>181</v>
       </c>
       <c r="B18" s="11"/>
       <c r="C18" s="19" t="n">
@@ -6315,7 +6323,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="13" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="B19" s="11"/>
       <c r="C19" s="20" t="n">
@@ -6355,8 +6363,8 @@
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="3" t="s">
-        <v>182</v>
+      <c r="A20" s="2" t="s">
+        <v>183</v>
       </c>
       <c r="B20" s="11"/>
       <c r="C20" s="19" t="n">
@@ -6402,12 +6410,12 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="21" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="13" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="B23" s="11"/>
       <c r="C23" s="16" t="n">
@@ -6445,13 +6453,13 @@
         <f aca="false">K23-(Assumptions!K63+Assumptions!L63)/Assumptions!$D$85/2</f>
         <v>257.655511</v>
       </c>
-      <c r="M23" s="2" t="s">
-        <v>185</v>
+      <c r="M23" s="3" t="s">
+        <v>186</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="3" t="s">
-        <v>186</v>
+      <c r="A24" s="2" t="s">
+        <v>187</v>
       </c>
       <c r="B24" s="11"/>
       <c r="C24" s="15" t="n">
@@ -6497,7 +6505,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="13" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="B25" s="11"/>
       <c r="C25" s="16" t="n">
@@ -6538,12 +6546,12 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="21" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="13" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="B28" s="11"/>
       <c r="C28" s="20" t="n">
@@ -6583,8 +6591,8 @@
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="3" t="s">
-        <v>190</v>
+      <c r="A29" s="2" t="s">
+        <v>191</v>
       </c>
       <c r="B29" s="11"/>
       <c r="C29" s="19" t="n">
@@ -6630,7 +6638,7 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="13" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="B30" s="11"/>
       <c r="C30" s="7" t="n">
@@ -6700,61 +6708,61 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
-        <v>193</v>
+      <c r="A2" s="3" t="s">
+        <v>194</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="9" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="B4" s="9"/>
       <c r="C4" s="10" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D4" s="10" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="E4" s="10" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="F4" s="10" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="G4" s="10" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="H4" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="I4" s="10" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="J4" s="10" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="K4" s="10" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="L4" s="10" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="M4" s="9" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="21" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="13" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="B7" s="11"/>
       <c r="C7" s="20" t="n">
@@ -6792,13 +6800,13 @@
         <f aca="false">CF!L35</f>
         <v>446706.782176175</v>
       </c>
-      <c r="M7" s="2" t="s">
-        <v>196</v>
+      <c r="M7" s="3" t="s">
+        <v>197</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="13" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="B8" s="11"/>
       <c r="C8" s="20" t="n">
@@ -6836,13 +6844,13 @@
         <f aca="false">K8</f>
         <v>33686</v>
       </c>
-      <c r="M8" s="2" t="s">
-        <v>197</v>
+      <c r="M8" s="3" t="s">
+        <v>198</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="13" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="B9" s="11"/>
       <c r="C9" s="20" t="n">
@@ -6883,7 +6891,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="13" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="B10" s="11"/>
       <c r="C10" s="20" t="n">
@@ -6924,7 +6932,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="13" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="B11" s="11"/>
       <c r="C11" s="20" t="n">
@@ -6964,8 +6972,8 @@
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="3" t="s">
-        <v>201</v>
+      <c r="A12" s="2" t="s">
+        <v>202</v>
       </c>
       <c r="B12" s="11"/>
       <c r="C12" s="19" t="n">
@@ -7011,7 +7019,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="13" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="B13" s="11"/>
       <c r="C13" s="20" t="n">
@@ -7049,13 +7057,13 @@
         <f aca="false">K13+CF!L38-CF!L8</f>
         <v>287859.867951794</v>
       </c>
-      <c r="M13" s="2" t="s">
-        <v>203</v>
+      <c r="M13" s="3" t="s">
+        <v>204</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="13" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="B14" s="11"/>
       <c r="C14" s="20" t="n">
@@ -7093,13 +7101,13 @@
         <f aca="false">K14</f>
         <v>9619</v>
       </c>
-      <c r="M14" s="2" t="s">
-        <v>197</v>
+      <c r="M14" s="3" t="s">
+        <v>198</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="13" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="B15" s="11"/>
       <c r="C15" s="20" t="n">
@@ -7137,13 +7145,13 @@
         <f aca="false">K15</f>
         <v>85308</v>
       </c>
-      <c r="M15" s="2" t="s">
-        <v>197</v>
+      <c r="M15" s="3" t="s">
+        <v>198</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="3" t="s">
-        <v>206</v>
+      <c r="A16" s="2" t="s">
+        <v>207</v>
       </c>
       <c r="B16" s="11"/>
       <c r="C16" s="19" t="n">
@@ -7188,8 +7196,8 @@
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="3" t="s">
-        <v>207</v>
+      <c r="A17" s="2" t="s">
+        <v>208</v>
       </c>
       <c r="B17" s="11"/>
       <c r="C17" s="19" t="n">
@@ -7235,12 +7243,12 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="21" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="13" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="B20" s="11"/>
       <c r="C20" s="20" t="n">
@@ -7281,7 +7289,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="13" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="B21" s="11"/>
       <c r="C21" s="20" t="n">
@@ -7319,13 +7327,13 @@
         <f aca="false">K21+CF!L27</f>
         <v>2384</v>
       </c>
-      <c r="M21" s="2" t="s">
-        <v>211</v>
+      <c r="M21" s="3" t="s">
+        <v>212</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="13" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="B22" s="11"/>
       <c r="C22" s="20" t="n">
@@ -7363,13 +7371,13 @@
         <f aca="false">K22</f>
         <v>20030</v>
       </c>
-      <c r="M22" s="2" t="s">
-        <v>197</v>
+      <c r="M22" s="3" t="s">
+        <v>198</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="13" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="B23" s="11"/>
       <c r="C23" s="20" t="n">
@@ -7410,7 +7418,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="13" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="B24" s="11"/>
       <c r="C24" s="20" t="n">
@@ -7448,13 +7456,13 @@
         <f aca="false">K24</f>
         <v>22498</v>
       </c>
-      <c r="M24" s="2" t="s">
-        <v>197</v>
+      <c r="M24" s="3" t="s">
+        <v>198</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="3" t="s">
-        <v>215</v>
+      <c r="A25" s="2" t="s">
+        <v>216</v>
       </c>
       <c r="B25" s="11"/>
       <c r="C25" s="19" t="n">
@@ -7500,12 +7508,12 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="21" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="13" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="B28" s="11"/>
       <c r="C28" s="20" t="n">
@@ -7546,7 +7554,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="13" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="B29" s="11"/>
       <c r="C29" s="20" t="n">
@@ -7587,7 +7595,7 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="13" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="B30" s="11"/>
       <c r="C30" s="20" t="n">
@@ -7628,7 +7636,7 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="13" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="B31" s="11"/>
       <c r="C31" s="20" t="n">
@@ -7666,13 +7674,13 @@
         <f aca="false">K31</f>
         <v>225342</v>
       </c>
-      <c r="M31" s="2" t="s">
-        <v>221</v>
+      <c r="M31" s="3" t="s">
+        <v>222</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="3" t="s">
-        <v>222</v>
+      <c r="A32" s="2" t="s">
+        <v>223</v>
       </c>
       <c r="B32" s="11"/>
       <c r="C32" s="19" t="n">
@@ -7718,7 +7726,7 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="13" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="B33" s="11"/>
       <c r="C33" s="20" t="n">
@@ -7758,8 +7766,8 @@
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="3" t="s">
-        <v>224</v>
+      <c r="A34" s="2" t="s">
+        <v>225</v>
       </c>
       <c r="B34" s="11"/>
       <c r="C34" s="19" t="n">
@@ -7804,8 +7812,8 @@
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="3" t="s">
-        <v>225</v>
+      <c r="A35" s="2" t="s">
+        <v>226</v>
       </c>
       <c r="B35" s="11"/>
       <c r="C35" s="19" t="n">
@@ -7851,7 +7859,7 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="13" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="B36" s="11"/>
       <c r="C36" s="27" t="n">
@@ -7894,18 +7902,18 @@
         <f aca="false">ROUND(L17-L35,3)</f>
         <v>1</v>
       </c>
-      <c r="M36" s="2" t="s">
-        <v>227</v>
+      <c r="M36" s="3" t="s">
+        <v>228</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="21" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="13" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="B39" s="11"/>
       <c r="C39" s="27" t="n">
@@ -7951,7 +7959,7 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="13" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="B40" s="11"/>
       <c r="C40" s="27" t="n">
@@ -7997,7 +8005,7 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="13" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="B41" s="11"/>
       <c r="C41" s="7" t="str">
@@ -8067,61 +8075,61 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
-        <v>232</v>
+      <c r="A2" s="3" t="s">
+        <v>233</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="9" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="B4" s="9"/>
       <c r="C4" s="10" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D4" s="10" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="E4" s="10" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="F4" s="10" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="G4" s="10" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="H4" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="I4" s="10" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="J4" s="10" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="K4" s="10" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="L4" s="10" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="M4" s="9" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="21" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="13" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="B7" s="11"/>
       <c r="C7" s="20" t="n">
@@ -8162,7 +8170,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="13" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="B8" s="11"/>
       <c r="H8" s="27" t="n">
@@ -8185,13 +8193,13 @@
         <f aca="false">Assumptions!$G$71*BS!K13</f>
         <v>26561.1219992585</v>
       </c>
-      <c r="M8" s="2" t="s">
-        <v>235</v>
+      <c r="M8" s="3" t="s">
+        <v>236</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="13" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="B9" s="11"/>
       <c r="H9" s="27" t="n">
@@ -8217,7 +8225,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="13" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="B10" s="11"/>
       <c r="C10" s="20" t="n">
@@ -8258,7 +8266,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="13" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="B11" s="11"/>
       <c r="C11" s="20" t="n">
@@ -8299,7 +8307,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="13" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="B12" s="11"/>
       <c r="C12" s="20" t="n">
@@ -8340,7 +8348,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="13" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="B13" s="11"/>
       <c r="C13" s="20" t="n">
@@ -8381,7 +8389,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="13" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="B14" s="11"/>
       <c r="H14" s="27" t="n">
@@ -8407,7 +8415,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="13" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="B15" s="11"/>
       <c r="C15" s="27" t="n">
@@ -8430,13 +8438,13 @@
         <f aca="false">G16-SUM(G7:G14)</f>
         <v>5041</v>
       </c>
-      <c r="M15" s="2" t="s">
-        <v>243</v>
+      <c r="M15" s="3" t="s">
+        <v>244</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="3" t="s">
-        <v>244</v>
+      <c r="A16" s="2" t="s">
+        <v>245</v>
       </c>
       <c r="B16" s="11"/>
       <c r="C16" s="31" t="n">
@@ -8474,18 +8482,18 @@
         <f aca="false">SUM(L7:L14)-L8-L9</f>
         <v>122748.003452432</v>
       </c>
-      <c r="M16" s="2" t="s">
-        <v>245</v>
+      <c r="M16" s="3" t="s">
+        <v>246</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="21" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="13" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="B19" s="11"/>
       <c r="C19" s="20" t="n">
@@ -8526,7 +8534,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="13" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="B20" s="11"/>
       <c r="C20" s="27" t="n">
@@ -8569,13 +8577,13 @@
         <f aca="false">0</f>
         <v>0</v>
       </c>
-      <c r="M20" s="2" t="s">
-        <v>249</v>
+      <c r="M20" s="3" t="s">
+        <v>250</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="3" t="s">
-        <v>250</v>
+      <c r="A21" s="2" t="s">
+        <v>251</v>
       </c>
       <c r="B21" s="11"/>
       <c r="C21" s="31" t="n">
@@ -8616,12 +8624,12 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="21" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="13" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="B24" s="11"/>
       <c r="C24" s="20" t="n">
@@ -8659,13 +8667,13 @@
         <f aca="false">-IS!L20*Assumptions!$G$76</f>
         <v>-48428.9805431481</v>
       </c>
-      <c r="M24" s="2" t="s">
-        <v>253</v>
+      <c r="M24" s="3" t="s">
+        <v>254</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="13" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="B25" s="11"/>
       <c r="C25" s="20" t="n">
@@ -8706,7 +8714,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="13" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="B26" s="11"/>
       <c r="C26" s="20" t="n">
@@ -8747,7 +8755,7 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="13" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="B27" s="11"/>
       <c r="C27" s="20" t="n">
@@ -8785,13 +8793,13 @@
         <f aca="false">MAX(0,Assumptions!$G$77-(L34+L16+L21+L24+L25+L26-(BS!K21-BS!G21)))-(BS!K21-BS!G21)</f>
         <v>0</v>
       </c>
-      <c r="M27" s="2" t="s">
-        <v>257</v>
+      <c r="M27" s="3" t="s">
+        <v>258</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="13" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="B28" s="11"/>
       <c r="C28" s="27" t="n">
@@ -8836,8 +8844,8 @@
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="3" t="s">
-        <v>259</v>
+      <c r="A29" s="2" t="s">
+        <v>260</v>
       </c>
       <c r="B29" s="11"/>
       <c r="C29" s="31" t="n">
@@ -8878,12 +8886,12 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="21" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="13" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="B32" s="11"/>
       <c r="C32" s="20" t="n">
@@ -8921,13 +8929,13 @@
         <f aca="false">0</f>
         <v>0</v>
       </c>
-      <c r="M32" s="2" t="s">
-        <v>262</v>
+      <c r="M32" s="3" t="s">
+        <v>263</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="3" t="s">
-        <v>263</v>
+      <c r="A33" s="2" t="s">
+        <v>264</v>
       </c>
       <c r="B33" s="11"/>
       <c r="C33" s="19" t="n">
@@ -8973,7 +8981,7 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="13" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="B34" s="11"/>
       <c r="C34" s="20" t="n">
@@ -9013,8 +9021,8 @@
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="3" t="s">
-        <v>265</v>
+      <c r="A35" s="2" t="s">
+        <v>266</v>
       </c>
       <c r="B35" s="11"/>
       <c r="C35" s="19" t="n">
@@ -9060,12 +9068,12 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="21" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="13" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="B38" s="11"/>
       <c r="C38" s="27" t="n">
@@ -9110,8 +9118,8 @@
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="3" t="s">
-        <v>267</v>
+      <c r="A39" s="2" t="s">
+        <v>268</v>
       </c>
       <c r="B39" s="11"/>
       <c r="C39" s="19" t="n">
@@ -9181,61 +9189,61 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
-        <v>269</v>
+      <c r="A2" s="3" t="s">
+        <v>270</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="9" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="B4" s="9"/>
       <c r="C4" s="10" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D4" s="10" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="E4" s="10" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="F4" s="10" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="G4" s="10" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="H4" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="I4" s="10" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="J4" s="10" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="K4" s="10" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="L4" s="10" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="M4" s="9" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="21" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="13" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="B7" s="11"/>
       <c r="H7" s="27" t="n">
@@ -9261,7 +9269,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="13" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="B8" s="11"/>
       <c r="H8" s="27" t="n">
@@ -9286,8 +9294,8 @@
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="3" t="s">
-        <v>273</v>
+      <c r="A9" s="2" t="s">
+        <v>274</v>
       </c>
       <c r="B9" s="11"/>
       <c r="H9" s="19" t="n">
@@ -9313,7 +9321,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="13" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="B10" s="11"/>
       <c r="H10" s="27" t="n">
@@ -9336,13 +9344,13 @@
         <f aca="false">CF!L8</f>
         <v>26561.1219992585</v>
       </c>
-      <c r="M10" s="2" t="s">
-        <v>275</v>
+      <c r="M10" s="3" t="s">
+        <v>276</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="13" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="B11" s="11"/>
       <c r="H11" s="27" t="n">
@@ -9368,7 +9376,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="13" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="B12" s="11"/>
       <c r="H12" s="27" t="n">
@@ -9393,8 +9401,8 @@
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="3" t="s">
-        <v>278</v>
+      <c r="A13" s="2" t="s">
+        <v>279</v>
       </c>
       <c r="B13" s="11"/>
       <c r="H13" s="19" t="n">
@@ -9420,7 +9428,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="13" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="B14" s="11"/>
       <c r="H14" s="7" t="n">
@@ -9446,12 +9454,12 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="21" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="13" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="B17" s="11"/>
       <c r="H17" s="32" t="n">
@@ -9477,7 +9485,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="13" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="B18" s="11"/>
       <c r="H18" s="32" t="n">
@@ -9503,7 +9511,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="13" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="B19" s="11"/>
       <c r="H19" s="28" t="n">
@@ -9529,7 +9537,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="13" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="B20" s="11"/>
       <c r="H20" s="28" t="n">
@@ -9555,7 +9563,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="13" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="B21" s="11"/>
       <c r="H21" s="27" t="n">
@@ -9581,7 +9589,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="13" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="B22" s="11"/>
       <c r="H22" s="28" t="n">
@@ -9606,8 +9614,8 @@
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="3" t="s">
-        <v>287</v>
+      <c r="A23" s="2" t="s">
+        <v>288</v>
       </c>
       <c r="B23" s="11"/>
       <c r="H23" s="19" t="n">
@@ -9633,7 +9641,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="13" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="B24" s="11"/>
       <c r="H24" s="30" t="n">
@@ -9659,24 +9667,24 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="21" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="13" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D27" s="7" t="n">
         <f aca="false">Assumptions!$D$101</f>
         <v>0.0883738674377037</v>
       </c>
-      <c r="M27" s="2" t="s">
-        <v>290</v>
+      <c r="M27" s="3" t="s">
+        <v>291</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="13" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="D28" s="7" t="n">
         <f aca="false">Assumptions!$G$78</f>
@@ -9685,7 +9693,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="13" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="D29" s="33" t="n">
         <f aca="false">Assumptions!$G$80</f>
@@ -9694,7 +9702,7 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="13" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="D30" s="28" t="n">
         <f aca="false">($L$18-Assumptions!$D$83)/365.25</f>
@@ -9703,7 +9711,7 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="13" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="D31" s="27" t="n">
         <f aca="false">SUM($H$23:$L$23)</f>
@@ -9712,24 +9720,24 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="13" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="D32" s="27" t="n">
         <f aca="false">Assumptions!$D$102+Assumptions!$D$103+Assumptions!$D$104-Assumptions!$D$105-Assumptions!$D$106-Assumptions!$D$108*Assumptions!$D$86</f>
         <v>310456.214631</v>
       </c>
-      <c r="M32" s="2" t="s">
-        <v>296</v>
+      <c r="M32" s="3" t="s">
+        <v>297</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="21" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="13" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="D35" s="7" t="n">
         <f aca="false">Assumptions!$G$79</f>
@@ -9738,19 +9746,19 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="13" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="D36" s="27" t="n">
         <f aca="false">$L$9*(1+DCF!$D$28)*(1-DCF!$D$28/DCF!$D$35)</f>
         <v>78230.5819388014</v>
       </c>
-      <c r="M36" s="2" t="s">
-        <v>300</v>
+      <c r="M36" s="3" t="s">
+        <v>301</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="13" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="D37" s="27" t="n">
         <f aca="false">DCF!$D$36/(DCF!$D$27-DCF!$D$28)</f>
@@ -9759,7 +9767,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="13" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="D38" s="27" t="n">
         <f aca="false">DCF!$D$37/(1+DCF!$D$27)^DCF!$D$30</f>
@@ -9768,7 +9776,7 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="13" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="D39" s="27" t="n">
         <f aca="false">DCF!$D$31+DCF!$D$38</f>
@@ -9777,7 +9785,7 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="13" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="D40" s="27" t="n">
         <f aca="false">DCF!$D$39+DCF!$D$32</f>
@@ -9785,8 +9793,8 @@
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="3" t="s">
-        <v>305</v>
+      <c r="A41" s="2" t="s">
+        <v>306</v>
       </c>
       <c r="D41" s="5" t="n">
         <f aca="false">DCF!$D$40/Assumptions!$D$86</f>
@@ -9795,7 +9803,7 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="13" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="D42" s="7" t="n">
         <f aca="false">DCF!$D$38/DCF!$D$39</f>
@@ -9804,36 +9812,36 @@
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="13" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="D43" s="33" t="n">
         <f aca="false">(DCF!$D$37+Assumptions!$D$107)/IS!$L$29</f>
         <v>7.3271093513078</v>
       </c>
-      <c r="M43" s="2" t="s">
-        <v>308</v>
+      <c r="M43" s="3" t="s">
+        <v>309</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="21" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="13" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="D46" s="27" t="n">
         <f aca="false">IS!$L$29*DCF!$D$29-Assumptions!$D$107</f>
         <v>1171607.47375604</v>
       </c>
-      <c r="M46" s="2" t="s">
-        <v>311</v>
+      <c r="M46" s="3" t="s">
+        <v>312</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="13" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="D47" s="27" t="n">
         <f aca="false">DCF!$D$46/(1+DCF!$D$27)^DCF!$D$30</f>
@@ -9842,7 +9850,7 @@
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="13" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="D48" s="27" t="n">
         <f aca="false">DCF!$D$31+DCF!$D$47</f>
@@ -9851,7 +9859,7 @@
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="13" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="D49" s="27" t="n">
         <f aca="false">DCF!$D$48+DCF!$D$32</f>
@@ -9859,8 +9867,8 @@
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A50" s="3" t="s">
-        <v>305</v>
+      <c r="A50" s="2" t="s">
+        <v>306</v>
       </c>
       <c r="D50" s="5" t="n">
         <f aca="false">DCF!$D$49/Assumptions!$D$86</f>
@@ -9869,24 +9877,24 @@
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="13" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="D51" s="7" t="n">
         <f aca="false">(-(($L$9/DCF!$D$35)-$L$9-DCF!$D$46)-SQRT(((($L$9/DCF!$D$35)-$L$9-DCF!$D$46))^2-4*($L$9/DCF!$D$35)*(DCF!$D$46*DCF!$D$27-$L$9)))/(2*$L$9/DCF!$D$35)</f>
         <v>0.0240544351411912</v>
       </c>
-      <c r="M51" s="2" t="s">
-        <v>313</v>
+      <c r="M51" s="3" t="s">
+        <v>314</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="21" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="13" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="D54" s="6" t="n">
         <f aca="false">AVERAGE(DCF!$D$41,DCF!$D$50)</f>
@@ -9895,7 +9903,7 @@
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="13" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D55" s="7" t="n">
         <f aca="false">Assumptions!$D$96</f>
@@ -9904,19 +9912,19 @@
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="13" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="D56" s="30" t="n">
         <f aca="false">(IS!$H$25-Assumptions!$D$108)+0.5*IS!$I$25</f>
         <v>165.392407277756</v>
       </c>
-      <c r="M56" s="2" t="s">
-        <v>317</v>
+      <c r="M56" s="3" t="s">
+        <v>318</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="13" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="D57" s="6" t="n">
         <f aca="false">DCF!$D$54*(1+DCF!$D$55)-DCF!$D$56</f>
@@ -9924,8 +9932,8 @@
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A58" s="3" t="s">
-        <v>319</v>
+      <c r="A58" s="2" t="s">
+        <v>320</v>
       </c>
       <c r="D58" s="5" t="n">
         <f aca="false">MROUND(DCF!$D$57,50)</f>
@@ -9934,7 +9942,7 @@
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="13" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="D59" s="6" t="n">
         <f aca="false">Assumptions!$D$85</f>
@@ -9942,8 +9950,8 @@
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A60" s="3" t="s">
-        <v>6</v>
+      <c r="A60" s="2" t="s">
+        <v>7</v>
       </c>
       <c r="D60" s="29" t="n">
         <f aca="false">DCF!$D$58/DCF!$D$59-1</f>
@@ -9952,7 +9960,7 @@
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="13" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="D61" s="7" t="n">
         <f aca="false">(DCF!$D$58+DCF!$D$56)/DCF!$D$59-1</f>
@@ -9960,15 +9968,15 @@
       </c>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A62" s="3" t="s">
-        <v>3</v>
+      <c r="A62" s="2" t="s">
+        <v>4</v>
       </c>
       <c r="D62" s="8" t="str">
         <f aca="false">IF(DCF!$D$60&gt;0.15,"BUY",IF(DCF!$D$60&lt;-0.1,"SELL","HOLD"))</f>
         <v>HOLD</v>
       </c>
-      <c r="M62" s="2" t="s">
-        <v>322</v>
+      <c r="M62" s="3" t="s">
+        <v>323</v>
       </c>
     </row>
   </sheetData>
@@ -9998,67 +10006,67 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
-        <v>324</v>
+      <c r="A2" s="3" t="s">
+        <v>325</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="9" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="D4" s="10" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="E4" s="10" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="F4" s="10" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="G4" s="10" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="H4" s="10" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="I4" s="10" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="J4" s="10" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="K4" s="10" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="L4" s="10" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="M4" s="10" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="N4" s="10" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="34" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="B5" s="34" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="C5" s="34" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="D5" s="20" t="n">
         <v>4807497.14264855</v>
@@ -10101,13 +10109,13 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="34" t="s">
+        <v>341</v>
+      </c>
+      <c r="B6" s="34" t="s">
+        <v>342</v>
+      </c>
+      <c r="C6" s="34" t="s">
         <v>340</v>
-      </c>
-      <c r="B6" s="34" t="s">
-        <v>341</v>
-      </c>
-      <c r="C6" s="34" t="s">
-        <v>339</v>
       </c>
       <c r="D6" s="20" t="n">
         <v>2425172.37357654</v>
@@ -10150,13 +10158,13 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="34" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="B7" s="34" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="C7" s="34" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="D7" s="20" t="n">
         <v>340370.657029525</v>
@@ -10199,13 +10207,13 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="34" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="B8" s="34" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="C8" s="34" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="D8" s="20" t="n">
         <v>236614.523186309</v>
@@ -10248,13 +10256,13 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="34" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="B9" s="34" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="C9" s="34" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="D9" s="20" t="n">
         <v>328577.762448</v>
@@ -10297,13 +10305,13 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="34" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="B10" s="34" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="C10" s="34" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="D10" s="20" t="n">
         <v>178038.01365</v>
@@ -10346,13 +10354,13 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="34" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="B11" s="34" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="C11" s="34" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="D11" s="20" t="n">
         <v>1574054.70409787</v>
@@ -10394,8 +10402,8 @@
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B12" s="3" t="s">
-        <v>354</v>
+      <c r="B12" s="2" t="s">
+        <v>355</v>
       </c>
       <c r="J12" s="23" t="n">
         <f aca="false">MEDIAN(J5:J11)</f>
@@ -10419,8 +10427,8 @@
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B13" s="3" t="s">
-        <v>355</v>
+      <c r="B13" s="2" t="s">
+        <v>356</v>
       </c>
       <c r="J13" s="23" t="n">
         <f aca="false">AVERAGE(J5:J11)</f>
@@ -10444,8 +10452,8 @@
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B14" s="3" t="s">
-        <v>356</v>
+      <c r="B14" s="2" t="s">
+        <v>357</v>
       </c>
       <c r="J14" s="23" t="n">
         <f aca="false">QUARTILE(J5:J11,1)</f>
@@ -10469,8 +10477,8 @@
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B15" s="3" t="s">
-        <v>357</v>
+      <c r="B15" s="2" t="s">
+        <v>358</v>
       </c>
       <c r="J15" s="23" t="n">
         <f aca="false">QUARTILE(J5:J11,3)</f>
@@ -10495,12 +10503,12 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="21" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B18" s="13" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="D18" s="27" t="n">
         <f aca="false">Assumptions!$D$92</f>
@@ -10509,30 +10517,30 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B19" s="13" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="D19" s="27" t="n">
         <f aca="false">Assumptions!$D$92+Assumptions!$D$91-Assumptions!$D$102-Assumptions!$D$103+Assumptions!$D$106</f>
         <v>1098593.399283</v>
       </c>
-      <c r="F19" s="2" t="s">
-        <v>361</v>
+      <c r="F19" s="3" t="s">
+        <v>362</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B20" s="13" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="D20" s="20" t="n">
         <v>797536</v>
       </c>
-      <c r="F20" s="2" t="s">
-        <v>363</v>
+      <c r="F20" s="3" t="s">
+        <v>364</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B21" s="13" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="D21" s="20" t="n">
         <v>140297</v>
@@ -10540,7 +10548,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B22" s="13" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="D22" s="20" t="n">
         <v>82999</v>
@@ -10548,7 +10556,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B23" s="13" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="D23" s="20" t="n">
         <v>1006541</v>
@@ -10556,7 +10564,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B24" s="13" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="D24" s="33" t="n">
         <f aca="false">Comps!$D$19/Comps!$D$21</f>
@@ -10565,7 +10573,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B25" s="13" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="D25" s="33" t="n">
         <f aca="false">Comps!$D$18/Comps!$D$22</f>
@@ -10574,7 +10582,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B26" s="13" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="D26" s="33" t="n">
         <f aca="false">Comps!$D$19/Comps!$D$20</f>
@@ -10583,7 +10591,7 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B27" s="13" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="D27" s="33" t="n">
         <f aca="false">Comps!$D$18/Comps!$D$23</f>
@@ -10592,18 +10600,18 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B28" s="13" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="D28" s="22" t="n">
         <v>9.79306499114322</v>
       </c>
-      <c r="F28" s="2" t="s">
-        <v>368</v>
+      <c r="F28" s="3" t="s">
+        <v>369</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B29" s="13" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="D29" s="22" t="n">
         <v>7.77181552965895</v>
@@ -10611,7 +10619,7 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B30" s="13" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="D30" s="22" t="n">
         <v>10.9137840348721</v>
@@ -10619,12 +10627,12 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="21" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B33" s="13" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="D33" s="6" t="n">
         <f aca="false">(Comps!$K$12*Comps!$D$21-Comps!$D$19+Comps!$D$18)/Assumptions!$D$86</f>
@@ -10633,7 +10641,7 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B34" s="13" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="D34" s="6" t="n">
         <f aca="false">Comps!$L$12*Comps!$D$22/Assumptions!$D$86</f>
@@ -10642,7 +10650,7 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B35" s="13" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="D35" s="6" t="n">
         <f aca="false">(Comps!$K$14*Comps!$D$21-Comps!$D$19+Comps!$D$18)/Assumptions!$D$86</f>
@@ -10651,7 +10659,7 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B36" s="13" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="D36" s="6" t="n">
         <f aca="false">Comps!$L$14*Comps!$D$22/Assumptions!$D$86</f>
@@ -10660,7 +10668,7 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B37" s="13" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="D37" s="6" t="n">
         <f aca="false">(Comps!$K$15*Comps!$D$21-Comps!$D$19+Comps!$D$18)/Assumptions!$D$86</f>
@@ -10669,7 +10677,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B38" s="13" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="D38" s="6" t="n">
         <f aca="false">Comps!$L$15*Comps!$D$22/Assumptions!$D$86</f>
@@ -10678,7 +10686,7 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B39" s="13" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="D39" s="6" t="n">
         <f aca="false">(Comps!$D$29*Comps!$D$21-Comps!$D$19+Comps!$D$18)/Assumptions!$D$86</f>
@@ -10687,7 +10695,7 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B40" s="13" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="D40" s="6" t="n">
         <f aca="false">(Comps!$D$30*Comps!$D$21-Comps!$D$19+Comps!$D$18)/Assumptions!$D$86</f>
@@ -10696,7 +10704,7 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B41" s="13" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="D41" s="6" t="n">
         <f aca="false">(Comps!$D$28*Comps!$D$21-Comps!$D$19+Comps!$D$18)/Assumptions!$D$86</f>
@@ -10704,8 +10712,8 @@
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B43" s="2" t="s">
-        <v>381</v>
+      <c r="B43" s="3" t="s">
+        <v>382</v>
       </c>
     </row>
   </sheetData>
@@ -10734,22 +10742,22 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
-        <v>383</v>
+      <c r="A2" s="3" t="s">
+        <v>384</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="21" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B5" s="11" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="C5" s="29" t="n">
         <f aca="false">DCF!$D$28+(-0.01)</f>
@@ -10904,12 +10912,12 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="21" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B13" s="11" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="C13" s="35" t="n">
         <f aca="false">DCF!$D$29+(-2)</f>
@@ -11064,12 +11072,12 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="21" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B21" s="11" t="s">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="C21" s="29" t="n">
         <f aca="false">0.11</f>
@@ -11223,8 +11231,8 @@
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="2" t="s">
-        <v>390</v>
+      <c r="A28" s="3" t="s">
+        <v>391</v>
       </c>
     </row>
   </sheetData>

</xml_diff>